<commit_message>
Spreadsheet page price cell, clickable links and tab footers in the .xlsx, cookieless download count, calculator link, stray URL redirect (#32)
The spreadsheet page's comparison table now matches the pricing card (free for 1 property; Schedule E report from $29/mo). The generated .xlsx carries real hyperlinks for the first time, with UTM-tagged app bridges on the Monthly Dashboard and Schedule E tabs. app.js sends a cookieless Vercel custom event for every download. The profit calculator links to the spreadsheet page in its text; the stray old spreadsheet URL redirects permanently; sitemap lastmod bumped.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017x1i612sijkvuTb3A5cZKa
</commit_message>
<xml_diff>
--- a/downloads/blackcat-airbnb-profit-tracker.xlsx
+++ b/downloads/blackcat-airbnb-profit-tracker.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="192">
   <si>
     <t>Black Cat Analytics — Airbnb Profit Tracker (updated Sept 2026 for the 15.5% host fee)</t>
   </si>
@@ -129,7 +129,7 @@
     <t>generates tax reports, and gives you AI-powered insights.</t>
   </si>
   <si>
-    <t>→ https://app.tryblackcat.com/signup?utm_source=tryblackcat&amp;utm_medium=spreadsheet&amp;utm_content=xlsx_instructions (Free to start)</t>
+    <t>→ Start free at app.tryblackcat.com (1 property, no card needed)</t>
   </si>
   <si>
     <t>Questions? support@tryblackcat.com</t>
@@ -381,6 +381,9 @@
     <t>Avg Revenue/Transaction</t>
   </si>
   <si>
+    <t>Black Cat builds this dashboard from your Airbnb export automatically. Free for 1 property →</t>
+  </si>
+  <si>
     <t>Black Cat Analytics — Per-Property Summary</t>
   </si>
   <si>
@@ -514,6 +517,9 @@
   </si>
   <si>
     <t>NET RENTAL INCOME (Line 21)</t>
+  </si>
+  <si>
+    <t>Black Cat prepares this Schedule E worksheet from your imported transactions. Starter plan, $29/mo, 14-day free trial →</t>
   </si>
   <si>
     <t>Black Cat Analytics — Cleaning Cost Tracker</t>
@@ -597,7 +603,7 @@
     <numFmt numFmtId="165" formatCode="$#,##0.00"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -620,6 +626,12 @@
       <b/>
       <color rgb="22C55E"/>
       <sz val="12"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <color rgb="FF1D4ED8"/>
+      <sz val="11"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -767,72 +779,73 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="10" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="165" fontId="9" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="8" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="8" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="9" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="166" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="8" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="8" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="9" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="9" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="12" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="13" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="165" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="165" fontId="8" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1604,7 +1617,7 @@
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A42" s="2" t="s">
+      <c r="A42" s="4" t="s">
         <v>37</v>
       </c>
     </row>
@@ -1619,6 +1632,9 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A42" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -1640,676 +1656,676 @@
   </cols>
   <sheetData>
     <row r="1" ht="48" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="6"/>
+      <c r="H2" s="6"/>
     </row>
     <row r="3" ht="8" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="G4" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="H4" s="7" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="D5" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="E5" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="F5" s="10">
+      <c r="F5" s="11">
         <v>1240</v>
       </c>
-      <c r="G5" s="9" t="s">
+      <c r="G5" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="H5" s="9" t="s">
+      <c r="H5" s="10" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="B6" s="12" t="s">
+      <c r="B6" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="C6" s="13" t="s">
+      <c r="C6" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="D6" s="13" t="s">
+      <c r="D6" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="E6" s="13" t="s">
+      <c r="E6" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="F6" s="14">
+      <c r="F6" s="15">
         <v>150</v>
       </c>
-      <c r="G6" s="13" t="s">
+      <c r="G6" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="H6" s="13" t="s">
+      <c r="H6" s="14" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="F7" s="10">
+      <c r="F7" s="11">
         <v>890</v>
       </c>
-      <c r="G7" s="9" t="s">
+      <c r="G7" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="H7" s="9" t="s">
+      <c r="H7" s="10" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="11" t="s">
+      <c r="A8" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="B8" s="12" t="s">
+      <c r="B8" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="C8" s="13" t="s">
+      <c r="C8" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="D8" s="13" t="s">
+      <c r="D8" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="E8" s="13" t="s">
+      <c r="E8" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="F8" s="14">
+      <c r="F8" s="15">
         <v>120</v>
       </c>
-      <c r="G8" s="13" t="s">
+      <c r="G8" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="H8" s="13" t="s">
+      <c r="H8" s="14" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="B9" s="15" t="s">
+      <c r="B9" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="C9" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="D9" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="F9" s="16">
+      <c r="F9" s="17">
         <v>45</v>
       </c>
-      <c r="G9" s="9" t="s">
+      <c r="G9" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="H9" s="9" t="s">
+      <c r="H9" s="10" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="11" t="s">
+      <c r="A10" s="12" t="s">
         <v>67</v>
       </c>
-      <c r="B10" s="17" t="s">
+      <c r="B10" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="C10" s="13" t="s">
+      <c r="C10" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="D10" s="13" t="s">
+      <c r="D10" s="14" t="s">
         <v>68</v>
       </c>
-      <c r="E10" s="13" t="s">
+      <c r="E10" s="14" t="s">
         <v>69</v>
       </c>
-      <c r="F10" s="18">
+      <c r="F10" s="19">
         <v>1560</v>
       </c>
-      <c r="G10" s="13" t="s">
+      <c r="G10" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="H10" s="13" t="s">
+      <c r="H10" s="14" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="7" t="s">
+      <c r="A11" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="B11" s="15" t="s">
+      <c r="B11" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="C11" s="9" t="s">
+      <c r="C11" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="D11" s="9" t="s">
+      <c r="D11" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="E11" s="9" t="s">
+      <c r="E11" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="F11" s="16">
+      <c r="F11" s="17">
         <v>180</v>
       </c>
-      <c r="G11" s="9" t="s">
+      <c r="G11" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="H11" s="9" t="s">
+      <c r="H11" s="10" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="11" t="s">
+      <c r="A12" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="B12" s="12" t="s">
+      <c r="B12" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="C12" s="13" t="s">
+      <c r="C12" s="14" t="s">
         <v>72</v>
       </c>
-      <c r="D12" s="13" t="s">
+      <c r="D12" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="E12" s="13" t="s">
+      <c r="E12" s="14" t="s">
         <v>73</v>
       </c>
-      <c r="F12" s="14">
+      <c r="F12" s="15">
         <v>340</v>
       </c>
-      <c r="G12" s="13" t="s">
+      <c r="G12" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="H12" s="13" t="s">
+      <c r="H12" s="14" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="7" t="s">
+      <c r="A13" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="B13" s="15" t="s">
+      <c r="B13" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="C13" s="9" t="s">
+      <c r="C13" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="D13" s="9" t="s">
+      <c r="D13" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="E13" s="9" t="s">
+      <c r="E13" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="F13" s="16">
+      <c r="F13" s="17">
         <v>225</v>
       </c>
-      <c r="G13" s="9" t="s">
+      <c r="G13" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="H13" s="9" t="s">
+      <c r="H13" s="10" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="11" t="s">
+      <c r="A14" s="12" t="s">
         <v>74</v>
       </c>
-      <c r="B14" s="12" t="s">
+      <c r="B14" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="C14" s="13" t="s">
+      <c r="C14" s="14" t="s">
         <v>75</v>
       </c>
-      <c r="D14" s="13" t="s">
+      <c r="D14" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="E14" s="13" t="s">
+      <c r="E14" s="14" t="s">
         <v>76</v>
       </c>
-      <c r="F14" s="14">
+      <c r="F14" s="15">
         <v>195</v>
       </c>
-      <c r="G14" s="13" t="s">
+      <c r="G14" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="H14" s="13" t="s">
+      <c r="H14" s="14" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="7" t="s">
+      <c r="A15" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="B15" s="15" t="s">
+      <c r="B15" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="C15" s="9" t="s">
+      <c r="C15" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="D15" s="9" t="s">
+      <c r="D15" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="E15" s="9" t="s">
+      <c r="E15" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="F15" s="16">
+      <c r="F15" s="17">
         <v>210</v>
       </c>
-      <c r="G15" s="9" t="s">
+      <c r="G15" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="H15" s="9" t="s">
+      <c r="H15" s="10" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" s="11" t="s">
+      <c r="A16" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="B16" s="17" t="s">
+      <c r="B16" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="C16" s="13" t="s">
+      <c r="C16" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="D16" s="13" t="s">
+      <c r="D16" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="E16" s="13" t="s">
+      <c r="E16" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="F16" s="18">
+      <c r="F16" s="19">
         <v>980</v>
       </c>
-      <c r="G16" s="13" t="s">
+      <c r="G16" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="H16" s="13" t="s">
+      <c r="H16" s="14" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="7" t="s">
+      <c r="A17" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="B17" s="15" t="s">
+      <c r="B17" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="C17" s="9" t="s">
+      <c r="C17" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="D17" s="9" t="s">
+      <c r="D17" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="E17" s="9" t="s">
+      <c r="E17" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="F17" s="16">
+      <c r="F17" s="17">
         <v>150</v>
       </c>
-      <c r="G17" s="9" t="s">
+      <c r="G17" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="H17" s="9" t="s">
+      <c r="H17" s="10" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="11" t="s">
+      <c r="A18" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="B18" s="12" t="s">
+      <c r="B18" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="C18" s="13" t="s">
+      <c r="C18" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="D18" s="13" t="s">
+      <c r="D18" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="E18" s="13" t="s">
+      <c r="E18" s="14" t="s">
         <v>83</v>
       </c>
-      <c r="F18" s="14">
+      <c r="F18" s="15">
         <v>185</v>
       </c>
-      <c r="G18" s="13" t="s">
+      <c r="G18" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="H18" s="13" t="s">
+      <c r="H18" s="14" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="7" t="s">
+      <c r="A19" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="B19" s="15" t="s">
+      <c r="B19" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="C19" s="9" t="s">
+      <c r="C19" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="D19" s="9" t="s">
+      <c r="D19" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="E19" s="9" t="s">
+      <c r="E19" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="F19" s="16">
+      <c r="F19" s="17">
         <v>210</v>
       </c>
-      <c r="G19" s="9" t="s">
+      <c r="G19" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="H19" s="9" t="s">
+      <c r="H19" s="10" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="11" t="s">
+      <c r="A20" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="B20" s="12" t="s">
+      <c r="B20" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="C20" s="13" t="s">
+      <c r="C20" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="D20" s="13" t="s">
+      <c r="D20" s="14" t="s">
         <v>68</v>
       </c>
-      <c r="E20" s="13" t="s">
+      <c r="E20" s="14" t="s">
         <v>84</v>
       </c>
-      <c r="F20" s="14">
+      <c r="F20" s="15">
         <v>195</v>
       </c>
-      <c r="G20" s="13" t="s">
+      <c r="G20" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="H20" s="13" t="s">
+      <c r="H20" s="14" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="7" t="s">
+      <c r="A21" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="B21" s="8" t="s">
+      <c r="B21" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="C21" s="9" t="s">
+      <c r="C21" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="D21" s="9" t="s">
+      <c r="D21" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="E21" s="9" t="s">
+      <c r="E21" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="F21" s="10">
+      <c r="F21" s="11">
         <v>2100</v>
       </c>
-      <c r="G21" s="9" t="s">
+      <c r="G21" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="H21" s="9" t="s">
+      <c r="H21" s="10" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="11" t="s">
+      <c r="A22" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="B22" s="12" t="s">
+      <c r="B22" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="C22" s="13" t="s">
+      <c r="C22" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="D22" s="13" t="s">
+      <c r="D22" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="E22" s="13" t="s">
+      <c r="E22" s="14" t="s">
         <v>87</v>
       </c>
-      <c r="F22" s="14">
+      <c r="F22" s="15">
         <v>140</v>
       </c>
-      <c r="G22" s="13" t="s">
+      <c r="G22" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="H22" s="13" t="s">
+      <c r="H22" s="14" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" s="7" t="s">
+      <c r="A23" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="B23" s="15" t="s">
+      <c r="B23" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="C23" s="9" t="s">
+      <c r="C23" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="D23" s="9" t="s">
+      <c r="D23" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="E23" s="9" t="s">
+      <c r="E23" s="10" t="s">
         <v>90</v>
       </c>
-      <c r="F23" s="16">
+      <c r="F23" s="17">
         <v>67</v>
       </c>
-      <c r="G23" s="9" t="s">
+      <c r="G23" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="H23" s="9" t="s">
+      <c r="H23" s="10" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" s="11" t="s">
+      <c r="A24" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="B24" s="12" t="s">
+      <c r="B24" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="C24" s="13" t="s">
+      <c r="C24" s="14" t="s">
         <v>89</v>
       </c>
-      <c r="D24" s="13" t="s">
+      <c r="D24" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="E24" s="13" t="s">
+      <c r="E24" s="14" t="s">
         <v>90</v>
       </c>
-      <c r="F24" s="14">
+      <c r="F24" s="15">
         <v>90</v>
       </c>
-      <c r="G24" s="13" t="s">
+      <c r="G24" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="H24" s="13" t="s">
+      <c r="H24" s="14" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A25" s="7" t="s">
+      <c r="A25" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="B25" s="15" t="s">
+      <c r="B25" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="C25" s="9" t="s">
+      <c r="C25" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="D25" s="9" t="s">
+      <c r="D25" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="E25" s="9" t="s">
+      <c r="E25" s="10" t="s">
         <v>90</v>
       </c>
-      <c r="F25" s="16">
+      <c r="F25" s="17">
         <v>47</v>
       </c>
-      <c r="G25" s="9" t="s">
+      <c r="G25" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="H25" s="9" t="s">
+      <c r="H25" s="10" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" s="11" t="s">
+      <c r="A26" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="B26" s="17" t="s">
+      <c r="B26" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="C26" s="13" t="s">
+      <c r="C26" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="D26" s="13" t="s">
+      <c r="D26" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="E26" s="13" t="s">
+      <c r="E26" s="14" t="s">
         <v>93</v>
       </c>
-      <c r="F26" s="18">
+      <c r="F26" s="19">
         <v>1000</v>
       </c>
-      <c r="G26" s="13" t="s">
+      <c r="G26" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="H26" s="13" t="s">
+      <c r="H26" s="14" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A27" s="7" t="s">
+      <c r="A27" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="B27" s="15" t="s">
+      <c r="B27" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="C27" s="9" t="s">
+      <c r="C27" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="D27" s="9" t="s">
+      <c r="D27" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="E27" s="9" t="s">
+      <c r="E27" s="10" t="s">
         <v>95</v>
       </c>
-      <c r="F27" s="16">
+      <c r="F27" s="17">
         <v>155</v>
       </c>
-      <c r="G27" s="9" t="s">
+      <c r="G27" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="H27" s="9" t="s">
+      <c r="H27" s="10" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A28" s="11" t="s">
+      <c r="A28" s="12" t="s">
         <v>97</v>
       </c>
-      <c r="B28" s="12" t="s">
+      <c r="B28" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="C28" s="13" t="s">
+      <c r="C28" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="D28" s="13" t="s">
+      <c r="D28" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="E28" s="13" t="s">
+      <c r="E28" s="14" t="s">
         <v>98</v>
       </c>
-      <c r="F28" s="14">
+      <c r="F28" s="15">
         <v>150</v>
       </c>
-      <c r="G28" s="13" t="s">
+      <c r="G28" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="H28" s="13" t="s">
+      <c r="H28" s="14" t="s">
         <v>1</v>
       </c>
     </row>
@@ -2818,7 +2834,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:N12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -2827,335 +2843,340 @@
   </cols>
   <sheetData>
     <row r="1" ht="48" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="6"/>
+      <c r="H2" s="6"/>
     </row>
     <row r="3" ht="8" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="20" t="s">
         <v>101</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="20" t="s">
         <v>102</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="D4" s="19" t="s">
+      <c r="D4" s="20" t="s">
         <v>104</v>
       </c>
-      <c r="E4" s="19" t="s">
+      <c r="E4" s="20" t="s">
         <v>105</v>
       </c>
-      <c r="F4" s="19" t="s">
+      <c r="F4" s="20" t="s">
         <v>106</v>
       </c>
-      <c r="G4" s="19" t="s">
+      <c r="G4" s="20" t="s">
         <v>107</v>
       </c>
-      <c r="H4" s="19" t="s">
+      <c r="H4" s="20" t="s">
         <v>108</v>
       </c>
-      <c r="I4" s="19" t="s">
+      <c r="I4" s="20" t="s">
         <v>109</v>
       </c>
-      <c r="J4" s="19" t="s">
+      <c r="J4" s="20" t="s">
         <v>110</v>
       </c>
-      <c r="K4" s="19" t="s">
+      <c r="K4" s="20" t="s">
         <v>111</v>
       </c>
-      <c r="L4" s="19" t="s">
+      <c r="L4" s="20" t="s">
         <v>112</v>
       </c>
-      <c r="M4" s="19" t="s">
+      <c r="M4" s="20" t="s">
         <v>113</v>
       </c>
-      <c r="N4" s="19" t="s">
+      <c r="N4" s="20" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A5" s="20" t="s">
+      <c r="A5" s="21" t="s">
         <v>115</v>
       </c>
-      <c r="B5" s="21">
+      <c r="B5" s="22">
         <f>SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=1)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Revenue")*'Revenue &amp; Expenses'!F5:F500)</f>
       </c>
-      <c r="C5" s="21">
+      <c r="C5" s="22">
         <f>SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=2)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Revenue")*'Revenue &amp; Expenses'!F5:F500)</f>
       </c>
-      <c r="D5" s="21">
+      <c r="D5" s="22">
         <f>SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=3)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Revenue")*'Revenue &amp; Expenses'!F5:F500)</f>
       </c>
-      <c r="E5" s="21">
+      <c r="E5" s="22">
         <f>SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=4)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Revenue")*'Revenue &amp; Expenses'!F5:F500)</f>
       </c>
-      <c r="F5" s="21">
+      <c r="F5" s="22">
         <f>SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=5)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Revenue")*'Revenue &amp; Expenses'!F5:F500)</f>
       </c>
-      <c r="G5" s="21">
+      <c r="G5" s="22">
         <f>SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=6)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Revenue")*'Revenue &amp; Expenses'!F5:F500)</f>
       </c>
-      <c r="H5" s="21">
+      <c r="H5" s="22">
         <f>SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=7)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Revenue")*'Revenue &amp; Expenses'!F5:F500)</f>
       </c>
-      <c r="I5" s="21">
+      <c r="I5" s="22">
         <f>SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=8)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Revenue")*'Revenue &amp; Expenses'!F5:F500)</f>
       </c>
-      <c r="J5" s="21">
+      <c r="J5" s="22">
         <f>SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=9)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Revenue")*'Revenue &amp; Expenses'!F5:F500)</f>
       </c>
-      <c r="K5" s="21">
+      <c r="K5" s="22">
         <f>SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=10)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Revenue")*'Revenue &amp; Expenses'!F5:F500)</f>
       </c>
-      <c r="L5" s="21">
+      <c r="L5" s="22">
         <f>SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=11)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Revenue")*'Revenue &amp; Expenses'!F5:F500)</f>
       </c>
-      <c r="M5" s="21">
+      <c r="M5" s="22">
         <f>SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=12)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Revenue")*'Revenue &amp; Expenses'!F5:F500)</f>
       </c>
-      <c r="N5" s="22">
+      <c r="N5" s="23">
         <f>SUM(B5:M5)</f>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A6" s="20" t="s">
+      <c r="A6" s="21" t="s">
         <v>116</v>
       </c>
-      <c r="B6" s="21">
+      <c r="B6" s="22">
         <f>SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=1)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Expense")*'Revenue &amp; Expenses'!F5:F500)</f>
       </c>
-      <c r="C6" s="21">
+      <c r="C6" s="22">
         <f>SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=2)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Expense")*'Revenue &amp; Expenses'!F5:F500)</f>
       </c>
-      <c r="D6" s="21">
+      <c r="D6" s="22">
         <f>SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=3)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Expense")*'Revenue &amp; Expenses'!F5:F500)</f>
       </c>
-      <c r="E6" s="21">
+      <c r="E6" s="22">
         <f>SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=4)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Expense")*'Revenue &amp; Expenses'!F5:F500)</f>
       </c>
-      <c r="F6" s="21">
+      <c r="F6" s="22">
         <f>SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=5)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Expense")*'Revenue &amp; Expenses'!F5:F500)</f>
       </c>
-      <c r="G6" s="21">
+      <c r="G6" s="22">
         <f>SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=6)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Expense")*'Revenue &amp; Expenses'!F5:F500)</f>
       </c>
-      <c r="H6" s="21">
+      <c r="H6" s="22">
         <f>SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=7)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Expense")*'Revenue &amp; Expenses'!F5:F500)</f>
       </c>
-      <c r="I6" s="21">
+      <c r="I6" s="22">
         <f>SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=8)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Expense")*'Revenue &amp; Expenses'!F5:F500)</f>
       </c>
-      <c r="J6" s="21">
+      <c r="J6" s="22">
         <f>SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=9)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Expense")*'Revenue &amp; Expenses'!F5:F500)</f>
       </c>
-      <c r="K6" s="21">
+      <c r="K6" s="22">
         <f>SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=10)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Expense")*'Revenue &amp; Expenses'!F5:F500)</f>
       </c>
-      <c r="L6" s="21">
+      <c r="L6" s="22">
         <f>SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=11)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Expense")*'Revenue &amp; Expenses'!F5:F500)</f>
       </c>
-      <c r="M6" s="21">
+      <c r="M6" s="22">
         <f>SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=12)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Expense")*'Revenue &amp; Expenses'!F5:F500)</f>
       </c>
-      <c r="N6" s="22">
+      <c r="N6" s="23">
         <f>SUM(B6:M6)</f>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A7" s="23" t="s">
+      <c r="A7" s="24" t="s">
         <v>117</v>
       </c>
-      <c r="B7" s="24">
+      <c r="B7" s="25">
         <f>B5-B6</f>
       </c>
-      <c r="C7" s="24">
+      <c r="C7" s="25">
         <f>C5-C6</f>
       </c>
-      <c r="D7" s="24">
+      <c r="D7" s="25">
         <f>D5-D6</f>
       </c>
-      <c r="E7" s="24">
+      <c r="E7" s="25">
         <f>E5-E6</f>
       </c>
-      <c r="F7" s="24">
+      <c r="F7" s="25">
         <f>F5-F6</f>
       </c>
-      <c r="G7" s="24">
+      <c r="G7" s="25">
         <f>G5-G6</f>
       </c>
-      <c r="H7" s="24">
+      <c r="H7" s="25">
         <f>H5-H6</f>
       </c>
-      <c r="I7" s="24">
+      <c r="I7" s="25">
         <f>I5-I6</f>
       </c>
-      <c r="J7" s="24">
+      <c r="J7" s="25">
         <f>J5-J6</f>
       </c>
-      <c r="K7" s="24">
+      <c r="K7" s="25">
         <f>K5-K6</f>
       </c>
-      <c r="L7" s="24">
+      <c r="L7" s="25">
         <f>L5-L6</f>
       </c>
-      <c r="M7" s="24">
+      <c r="M7" s="25">
         <f>M5-M6</f>
       </c>
-      <c r="N7" s="24">
+      <c r="N7" s="25">
         <f>SUM(B7:M7)</f>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" s="20" t="s">
+      <c r="A8" s="21" t="s">
         <v>118</v>
       </c>
-      <c r="B8" s="25">
+      <c r="B8" s="26">
         <f>IF(B5=0,0,B7/B5)</f>
       </c>
-      <c r="C8" s="25">
+      <c r="C8" s="26">
         <f>IF(C5=0,0,C7/C5)</f>
       </c>
-      <c r="D8" s="25">
+      <c r="D8" s="26">
         <f>IF(D5=0,0,D7/D5)</f>
       </c>
-      <c r="E8" s="25">
+      <c r="E8" s="26">
         <f>IF(E5=0,0,E7/E5)</f>
       </c>
-      <c r="F8" s="25">
+      <c r="F8" s="26">
         <f>IF(F5=0,0,F7/F5)</f>
       </c>
-      <c r="G8" s="25">
+      <c r="G8" s="26">
         <f>IF(G5=0,0,G7/G5)</f>
       </c>
-      <c r="H8" s="25">
+      <c r="H8" s="26">
         <f>IF(H5=0,0,H7/H5)</f>
       </c>
-      <c r="I8" s="25">
+      <c r="I8" s="26">
         <f>IF(I5=0,0,I7/I5)</f>
       </c>
-      <c r="J8" s="25">
+      <c r="J8" s="26">
         <f>IF(J5=0,0,J7/J5)</f>
       </c>
-      <c r="K8" s="25">
+      <c r="K8" s="26">
         <f>IF(K5=0,0,K7/K5)</f>
       </c>
-      <c r="L8" s="25">
+      <c r="L8" s="26">
         <f>IF(L5=0,0,L7/L5)</f>
       </c>
-      <c r="M8" s="25">
+      <c r="M8" s="26">
         <f>IF(M5=0,0,M7/M5)</f>
       </c>
-      <c r="N8" s="26">
+      <c r="N8" s="27">
         <f>IF(N5=0,0,N7/N5)</f>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A9" s="20" t="s">
+      <c r="A9" s="21" t="s">
         <v>119</v>
       </c>
-      <c r="B9" s="9">
+      <c r="B9" s="10">
         <f>SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=1)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500&lt;&gt;""))</f>
       </c>
-      <c r="C9" s="9">
+      <c r="C9" s="10">
         <f>SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=2)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500&lt;&gt;""))</f>
       </c>
-      <c r="D9" s="9">
+      <c r="D9" s="10">
         <f>SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=3)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500&lt;&gt;""))</f>
       </c>
-      <c r="E9" s="9">
+      <c r="E9" s="10">
         <f>SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=4)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500&lt;&gt;""))</f>
       </c>
-      <c r="F9" s="9">
+      <c r="F9" s="10">
         <f>SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=5)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500&lt;&gt;""))</f>
       </c>
-      <c r="G9" s="9">
+      <c r="G9" s="10">
         <f>SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=6)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500&lt;&gt;""))</f>
       </c>
-      <c r="H9" s="9">
+      <c r="H9" s="10">
         <f>SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=7)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500&lt;&gt;""))</f>
       </c>
-      <c r="I9" s="9">
+      <c r="I9" s="10">
         <f>SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=8)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500&lt;&gt;""))</f>
       </c>
-      <c r="J9" s="9">
+      <c r="J9" s="10">
         <f>SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=9)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500&lt;&gt;""))</f>
       </c>
-      <c r="K9" s="9">
+      <c r="K9" s="10">
         <f>SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=10)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500&lt;&gt;""))</f>
       </c>
-      <c r="L9" s="9">
+      <c r="L9" s="10">
         <f>SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=11)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500&lt;&gt;""))</f>
       </c>
-      <c r="M9" s="9">
+      <c r="M9" s="10">
         <f>SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=12)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500&lt;&gt;""))</f>
       </c>
-      <c r="N9" s="20">
+      <c r="N9" s="21">
         <f>SUM(B9:M9)</f>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A10" s="20" t="s">
+      <c r="A10" s="21" t="s">
         <v>120</v>
       </c>
-      <c r="B10" s="21">
+      <c r="B10" s="22">
         <f>IF(SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=1)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Revenue"))=0,0,B5/SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=1)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Revenue")))</f>
       </c>
-      <c r="C10" s="21">
+      <c r="C10" s="22">
         <f>IF(SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=2)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Revenue"))=0,0,C5/SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=2)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Revenue")))</f>
       </c>
-      <c r="D10" s="21">
+      <c r="D10" s="22">
         <f>IF(SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=3)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Revenue"))=0,0,D5/SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=3)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Revenue")))</f>
       </c>
-      <c r="E10" s="21">
+      <c r="E10" s="22">
         <f>IF(SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=4)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Revenue"))=0,0,E5/SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=4)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Revenue")))</f>
       </c>
-      <c r="F10" s="21">
+      <c r="F10" s="22">
         <f>IF(SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=5)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Revenue"))=0,0,F5/SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=5)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Revenue")))</f>
       </c>
-      <c r="G10" s="21">
+      <c r="G10" s="22">
         <f>IF(SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=6)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Revenue"))=0,0,G5/SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=6)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Revenue")))</f>
       </c>
-      <c r="H10" s="21">
+      <c r="H10" s="22">
         <f>IF(SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=7)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Revenue"))=0,0,H5/SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=7)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Revenue")))</f>
       </c>
-      <c r="I10" s="21">
+      <c r="I10" s="22">
         <f>IF(SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=8)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Revenue"))=0,0,I5/SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=8)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Revenue")))</f>
       </c>
-      <c r="J10" s="21">
+      <c r="J10" s="22">
         <f>IF(SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=9)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Revenue"))=0,0,J5/SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=9)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Revenue")))</f>
       </c>
-      <c r="K10" s="21">
+      <c r="K10" s="22">
         <f>IF(SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=10)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Revenue"))=0,0,K5/SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=10)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Revenue")))</f>
       </c>
-      <c r="L10" s="21">
+      <c r="L10" s="22">
         <f>IF(SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=11)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Revenue"))=0,0,L5/SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=11)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Revenue")))</f>
       </c>
-      <c r="M10" s="21">
+      <c r="M10" s="22">
         <f>IF(SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=12)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Revenue"))=0,0,M5/SUMPRODUCT((MONTH('Revenue &amp; Expenses'!A5:A500)=12)*(YEAR('Revenue &amp; Expenses'!A5:A500)=2026)*('Revenue &amp; Expenses'!B5:B500="Revenue")))</f>
       </c>
-      <c r="N10" s="22">
+      <c r="N10" s="23">
         <f>IF(N9=0,0,N5/N9)</f>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>121</v>
       </c>
     </row>
   </sheetData>
@@ -3163,9 +3184,12 @@
     <mergeCell ref="B1:H1"/>
     <mergeCell ref="A2:H2"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="A12" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-  <drawing r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -3183,148 +3207,148 @@
   </cols>
   <sheetData>
     <row r="1" ht="48" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B1" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
+      <c r="B1" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
+      <c r="A2" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="6"/>
+      <c r="H2" s="6"/>
     </row>
     <row r="3" ht="8" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="27" t="s">
-        <v>123</v>
-      </c>
-      <c r="B4" s="27" t="s">
+      <c r="A4" s="28" t="s">
+        <v>124</v>
+      </c>
+      <c r="B4" s="28" t="s">
         <v>115</v>
       </c>
-      <c r="C4" s="27" t="s">
+      <c r="C4" s="28" t="s">
         <v>116</v>
       </c>
-      <c r="D4" s="27" t="s">
+      <c r="D4" s="28" t="s">
         <v>117</v>
       </c>
-      <c r="E4" s="27" t="s">
+      <c r="E4" s="28" t="s">
         <v>118</v>
       </c>
-      <c r="F4" s="27" t="s">
-        <v>124</v>
-      </c>
-      <c r="G4" s="27" t="s">
+      <c r="F4" s="28" t="s">
         <v>125</v>
       </c>
-      <c r="H4" s="27" t="s">
+      <c r="G4" s="28" t="s">
         <v>126</v>
       </c>
+      <c r="H4" s="28" t="s">
+        <v>127</v>
+      </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="20" t="s">
+      <c r="A5" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="B5" s="28">
+      <c r="B5" s="29">
         <f>SUMPRODUCT(('Revenue &amp; Expenses'!D5:D500="Downtown Loft")*('Revenue &amp; Expenses'!B5:B500="Revenue")*'Revenue &amp; Expenses'!F5:F500)</f>
       </c>
-      <c r="C5" s="28">
+      <c r="C5" s="29">
         <f>SUMPRODUCT(('Revenue &amp; Expenses'!D5:D500="Downtown Loft")*('Revenue &amp; Expenses'!B5:B500="Expense")*'Revenue &amp; Expenses'!F5:F500)</f>
       </c>
-      <c r="D5" s="10">
+      <c r="D5" s="11">
         <f>B5-C5</f>
       </c>
-      <c r="E5" s="29">
+      <c r="E5" s="30">
         <f>IF(B5=0,0,D5/B5)</f>
       </c>
       <c r="F5">
         <f>SUMPRODUCT(('Revenue &amp; Expenses'!D5:D500="Downtown Loft")*('Revenue &amp; Expenses'!B5:B500="Revenue"))</f>
       </c>
-      <c r="G5" s="28">
+      <c r="G5" s="29">
         <f>IF(F5=0,0,B5/F5)</f>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="30" t="s">
+      <c r="A6" s="31" t="s">
         <v>61</v>
       </c>
-      <c r="B6" s="31">
+      <c r="B6" s="32">
         <f>SUMPRODUCT(('Revenue &amp; Expenses'!D5:D500="Lakeside Cabin")*('Revenue &amp; Expenses'!B5:B500="Revenue")*'Revenue &amp; Expenses'!F5:F500)</f>
       </c>
-      <c r="C6" s="31">
+      <c r="C6" s="32">
         <f>SUMPRODUCT(('Revenue &amp; Expenses'!D5:D500="Lakeside Cabin")*('Revenue &amp; Expenses'!B5:B500="Expense")*'Revenue &amp; Expenses'!F5:F500)</f>
       </c>
-      <c r="D6" s="18">
+      <c r="D6" s="19">
         <f>B6-C6</f>
       </c>
-      <c r="E6" s="32">
+      <c r="E6" s="33">
         <f>IF(B6=0,0,D6/B6)</f>
       </c>
-      <c r="F6" s="33">
+      <c r="F6" s="34">
         <f>SUMPRODUCT(('Revenue &amp; Expenses'!D5:D500="Lakeside Cabin")*('Revenue &amp; Expenses'!B5:B500="Revenue"))</f>
       </c>
-      <c r="G6" s="31">
+      <c r="G6" s="32">
         <f>IF(F6=0,0,B6/F6)</f>
       </c>
-      <c r="H6" s="33"/>
+      <c r="H6" s="34"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="20" t="s">
+      <c r="A7" s="21" t="s">
         <v>68</v>
       </c>
-      <c r="B7" s="28">
+      <c r="B7" s="29">
         <f>SUMPRODUCT(('Revenue &amp; Expenses'!D5:D500="Beach Bungalow")*('Revenue &amp; Expenses'!B5:B500="Revenue")*'Revenue &amp; Expenses'!F5:F500)</f>
       </c>
-      <c r="C7" s="28">
+      <c r="C7" s="29">
         <f>SUMPRODUCT(('Revenue &amp; Expenses'!D5:D500="Beach Bungalow")*('Revenue &amp; Expenses'!B5:B500="Expense")*'Revenue &amp; Expenses'!F5:F500)</f>
       </c>
-      <c r="D7" s="10">
+      <c r="D7" s="11">
         <f>B7-C7</f>
       </c>
-      <c r="E7" s="29">
+      <c r="E7" s="30">
         <f>IF(B7=0,0,D7/B7)</f>
       </c>
       <c r="F7">
         <f>SUMPRODUCT(('Revenue &amp; Expenses'!D5:D500="Beach Bungalow")*('Revenue &amp; Expenses'!B5:B500="Revenue"))</f>
       </c>
-      <c r="G7" s="28">
+      <c r="G7" s="29">
         <f>IF(F7=0,0,B7/F7)</f>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="34" t="s">
-        <v>127</v>
-      </c>
-      <c r="B8" s="35">
+      <c r="A8" s="35" t="s">
+        <v>128</v>
+      </c>
+      <c r="B8" s="36">
         <f>SUM(B5:B7)</f>
       </c>
-      <c r="C8" s="35">
+      <c r="C8" s="36">
         <f>SUM(C5:C7)</f>
       </c>
-      <c r="D8" s="35">
+      <c r="D8" s="36">
         <f>SUM(D5:D7)</f>
       </c>
-      <c r="E8" s="36">
+      <c r="E8" s="37">
         <f>IF(B8=0,0,D8/B8)</f>
       </c>
-      <c r="F8" s="34">
+      <c r="F8" s="35">
         <f>SUM(F5:F7)</f>
       </c>
-      <c r="G8" s="35">
+      <c r="G8" s="36">
         <f>IF(F8=0,0,B8/F8)</f>
       </c>
-      <c r="H8" s="34"/>
+      <c r="H8" s="35"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3339,7 +3363,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -3349,293 +3373,298 @@
   </cols>
   <sheetData>
     <row r="1" ht="48" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B1" s="4" t="s">
-        <v>128</v>
-      </c>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
+      <c r="B1" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
-        <v>129</v>
-      </c>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
+      <c r="A2" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="6"/>
+      <c r="H2" s="6"/>
     </row>
     <row r="3" ht="8" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" s="37" t="s">
-        <v>130</v>
+      <c r="A4" s="38" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="5" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B5" s="9" t="s">
-        <v>131</v>
-      </c>
-      <c r="C5" s="20">
+      <c r="B5" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="C5" s="21">
         <v>2026</v>
       </c>
     </row>
     <row r="6" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B6" s="9" t="s">
-        <v>132</v>
-      </c>
-      <c r="C6" s="20">
+      <c r="B6" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="C6" s="21">
         <v>280</v>
       </c>
     </row>
     <row r="7" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B7" s="9" t="s">
-        <v>133</v>
-      </c>
-      <c r="C7" s="20">
+      <c r="B7" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="C7" s="21">
         <v>30</v>
       </c>
     </row>
     <row r="8" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B8" s="9" t="s">
-        <v>134</v>
-      </c>
-      <c r="C8" s="26">
+      <c r="B8" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="C8" s="27">
         <f>C6/(C6+C7)</f>
       </c>
     </row>
     <row r="10" ht="8" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="11" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="38" t="s">
-        <v>135</v>
-      </c>
-      <c r="B11" s="38" t="s">
+      <c r="A11" s="39" t="s">
         <v>136</v>
       </c>
-      <c r="C11" s="38" t="s">
+      <c r="B11" s="39" t="s">
         <v>137</v>
       </c>
-      <c r="D11" s="38" t="s">
+      <c r="C11" s="39" t="s">
         <v>138</v>
       </c>
-      <c r="E11" s="38" t="s">
+      <c r="D11" s="39" t="s">
         <v>139</v>
       </c>
+      <c r="E11" s="39" t="s">
+        <v>140</v>
+      </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="39" t="s">
-        <v>140</v>
-      </c>
-      <c r="B12" s="9" t="s">
+      <c r="A12" s="40" t="s">
         <v>141</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="B12" s="10" t="s">
         <v>142</v>
       </c>
-      <c r="D12" s="28">
+      <c r="C12" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="D12" s="29">
         <f>SUMPRODUCT(('Revenue &amp; Expenses'!C5:C500="Airbnb Payout")*('Revenue &amp; Expenses'!B5:B500="Revenue")*'Revenue &amp; Expenses'!F5:F500)+SUMPRODUCT(('Revenue &amp; Expenses'!C5:C500="VRBO Payout")*('Revenue &amp; Expenses'!B5:B500="Revenue")*'Revenue &amp; Expenses'!F5:F500)+SUMPRODUCT(('Revenue &amp; Expenses'!C5:C500="Other Revenue")*('Revenue &amp; Expenses'!B5:B500="Revenue")*'Revenue &amp; Expenses'!F5:F500)</f>
       </c>
-      <c r="E12" s="28">
+      <c r="E12" s="29">
         <f>D12</f>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="40" t="s">
-        <v>143</v>
-      </c>
-      <c r="B13" s="13" t="s">
+      <c r="A13" s="41" t="s">
         <v>144</v>
       </c>
-      <c r="C13" s="41" t="s">
-        <v>144</v>
-      </c>
-      <c r="D13" s="31">
+      <c r="B13" s="14" t="s">
+        <v>145</v>
+      </c>
+      <c r="C13" s="42" t="s">
+        <v>145</v>
+      </c>
+      <c r="D13" s="32">
         <f>SUMPRODUCT(('Revenue &amp; Expenses'!C5:C500="Advertising")*('Revenue &amp; Expenses'!B5:B500="Expense")*'Revenue &amp; Expenses'!F5:F500)</f>
       </c>
-      <c r="E13" s="31">
+      <c r="E13" s="32">
         <f>D13</f>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="39" t="s">
-        <v>145</v>
-      </c>
-      <c r="B14" s="9" t="s">
+      <c r="A14" s="40" t="s">
         <v>146</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="B14" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="C14" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="D14" s="28">
+      <c r="D14" s="29">
         <f>SUMPRODUCT(('Revenue &amp; Expenses'!C5:C500="Cleaning")*('Revenue &amp; Expenses'!B5:B500="Expense")*'Revenue &amp; Expenses'!F5:F500)</f>
       </c>
-      <c r="E14" s="28">
+      <c r="E14" s="29">
         <f>D14</f>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="40" t="s">
-        <v>147</v>
-      </c>
-      <c r="B15" s="13" t="s">
+      <c r="A15" s="41" t="s">
         <v>148</v>
       </c>
-      <c r="C15" s="41" t="s">
+      <c r="B15" s="14" t="s">
         <v>149</v>
       </c>
-      <c r="D15" s="31">
+      <c r="C15" s="42" t="s">
+        <v>150</v>
+      </c>
+      <c r="D15" s="32">
         <f>SUMPRODUCT(('Revenue &amp; Expenses'!C5:C500="Platform Fees")*('Revenue &amp; Expenses'!B5:B500="Expense")*'Revenue &amp; Expenses'!F5:F500)+SUMPRODUCT(('Revenue &amp; Expenses'!C5:C500="Management Fees")*('Revenue &amp; Expenses'!B5:B500="Expense")*'Revenue &amp; Expenses'!F5:F500)</f>
       </c>
-      <c r="E15" s="31">
+      <c r="E15" s="32">
         <f>D15</f>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="39" t="s">
-        <v>150</v>
-      </c>
-      <c r="B16" s="9" t="s">
+      <c r="A16" s="40" t="s">
+        <v>151</v>
+      </c>
+      <c r="B16" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="C16" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="D16" s="28">
+      <c r="D16" s="29">
         <f>SUMPRODUCT(('Revenue &amp; Expenses'!C5:C500="Insurance")*('Revenue &amp; Expenses'!B5:B500="Expense")*'Revenue &amp; Expenses'!F5:F500)</f>
       </c>
-      <c r="E16" s="28">
+      <c r="E16" s="29">
         <f>D16*$C$8</f>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="40" t="s">
-        <v>151</v>
-      </c>
-      <c r="B17" s="13" t="s">
+      <c r="A17" s="41" t="s">
         <v>152</v>
       </c>
-      <c r="C17" s="41" t="s">
-        <v>152</v>
-      </c>
-      <c r="D17" s="31">
+      <c r="B17" s="14" t="s">
+        <v>153</v>
+      </c>
+      <c r="C17" s="42" t="s">
+        <v>153</v>
+      </c>
+      <c r="D17" s="32">
         <f>SUMPRODUCT(('Revenue &amp; Expenses'!C5:C500="Mortgage Interest")*('Revenue &amp; Expenses'!B5:B500="Expense")*'Revenue &amp; Expenses'!F5:F500)</f>
       </c>
-      <c r="E17" s="31">
+      <c r="E17" s="32">
         <f>D17*$C$8</f>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="39" t="s">
-        <v>153</v>
-      </c>
-      <c r="B18" s="9" t="s">
+      <c r="A18" s="40" t="s">
         <v>154</v>
       </c>
-      <c r="C18" s="5" t="s">
+      <c r="B18" s="10" t="s">
+        <v>155</v>
+      </c>
+      <c r="C18" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="D18" s="28">
+      <c r="D18" s="29">
         <f>SUMPRODUCT(('Revenue &amp; Expenses'!C5:C500="Maintenance &amp; Repairs")*('Revenue &amp; Expenses'!B5:B500="Expense")*'Revenue &amp; Expenses'!F5:F500)</f>
       </c>
-      <c r="E18" s="28">
+      <c r="E18" s="29">
         <f>D18*$C$8</f>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="40" t="s">
-        <v>155</v>
-      </c>
-      <c r="B19" s="13" t="s">
+      <c r="A19" s="41" t="s">
         <v>156</v>
       </c>
-      <c r="C19" s="41" t="s">
+      <c r="B19" s="14" t="s">
         <v>157</v>
       </c>
-      <c r="D19" s="31">
+      <c r="C19" s="42" t="s">
+        <v>158</v>
+      </c>
+      <c r="D19" s="32">
         <f>SUMPRODUCT(('Revenue &amp; Expenses'!C5:C500="Property Tax")*('Revenue &amp; Expenses'!B5:B500="Expense")*'Revenue &amp; Expenses'!F5:F500)</f>
       </c>
-      <c r="E19" s="31">
+      <c r="E19" s="32">
         <f>D19*$C$8</f>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="39" t="s">
-        <v>158</v>
-      </c>
-      <c r="B20" s="9" t="s">
+      <c r="A20" s="40" t="s">
+        <v>159</v>
+      </c>
+      <c r="B20" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="C20" s="5" t="s">
+      <c r="C20" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="D20" s="28">
+      <c r="D20" s="29">
         <f>SUMPRODUCT(('Revenue &amp; Expenses'!C5:C500="Utilities")*('Revenue &amp; Expenses'!B5:B500="Expense")*'Revenue &amp; Expenses'!F5:F500)</f>
       </c>
-      <c r="E20" s="28">
+      <c r="E20" s="29">
         <f>D20*$C$8</f>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="40" t="s">
-        <v>159</v>
-      </c>
-      <c r="B21" s="13" t="s">
+      <c r="A21" s="41" t="s">
         <v>160</v>
       </c>
-      <c r="C21" s="41" t="s">
-        <v>160</v>
-      </c>
-      <c r="D21" s="31">
+      <c r="B21" s="14" t="s">
+        <v>161</v>
+      </c>
+      <c r="C21" s="42" t="s">
+        <v>161</v>
+      </c>
+      <c r="D21" s="32">
         <f>SUMPRODUCT(('Revenue &amp; Expenses'!C5:C500="Depreciation")*('Revenue &amp; Expenses'!B5:B500="Expense")*'Revenue &amp; Expenses'!F5:F500)</f>
       </c>
-      <c r="E21" s="31">
+      <c r="E21" s="32">
         <f>D21*$C$8</f>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="39" t="s">
-        <v>161</v>
-      </c>
-      <c r="B22" s="9" t="s">
+      <c r="A22" s="40" t="s">
         <v>162</v>
       </c>
-      <c r="C22" s="5" t="s">
+      <c r="B22" s="10" t="s">
         <v>163</v>
       </c>
-      <c r="D22" s="28">
+      <c r="C22" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="D22" s="29">
         <f>SUMPRODUCT(('Revenue &amp; Expenses'!C5:C500="Supplies")*('Revenue &amp; Expenses'!B5:B500="Expense")*'Revenue &amp; Expenses'!F5:F500)+SUMPRODUCT(('Revenue &amp; Expenses'!C5:C500="Other Expense")*('Revenue &amp; Expenses'!B5:B500="Expense")*'Revenue &amp; Expenses'!F5:F500)</f>
       </c>
-      <c r="E22" s="28">
+      <c r="E22" s="29">
         <f>D22</f>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="42"/>
-      <c r="B23" s="42" t="s">
-        <v>164</v>
-      </c>
-      <c r="C23" s="42"/>
-      <c r="D23" s="43">
+      <c r="A23" s="43"/>
+      <c r="B23" s="43" t="s">
+        <v>165</v>
+      </c>
+      <c r="C23" s="43"/>
+      <c r="D23" s="44">
         <f>SUM(D13:D22)</f>
       </c>
-      <c r="E23" s="43">
+      <c r="E23" s="44">
         <f>SUM(E13:E22)</f>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" s="44"/>
-      <c r="B24" s="44" t="s">
-        <v>165</v>
-      </c>
-      <c r="C24" s="44"/>
-      <c r="D24" s="44"/>
-      <c r="E24" s="45">
+      <c r="A24" s="45"/>
+      <c r="B24" s="45" t="s">
+        <v>166</v>
+      </c>
+      <c r="C24" s="45"/>
+      <c r="D24" s="45"/>
+      <c r="E24" s="46">
         <f>E12-E23</f>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" s="4" t="s">
+        <v>167</v>
       </c>
     </row>
   </sheetData>
@@ -3643,9 +3672,12 @@
     <mergeCell ref="B1:H1"/>
     <mergeCell ref="A2:H2"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="A26" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-  <drawing r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -3665,247 +3697,247 @@
   </cols>
   <sheetData>
     <row r="1" ht="48" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B1" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
+      <c r="B1" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
-        <v>167</v>
-      </c>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
+      <c r="A2" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="6"/>
+      <c r="H2" s="6"/>
     </row>
     <row r="3" ht="8" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" ht="28" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="46" t="s">
+      <c r="A4" s="47" t="s">
         <v>41</v>
       </c>
-      <c r="B4" s="46" t="s">
+      <c r="B4" s="47" t="s">
         <v>44</v>
       </c>
-      <c r="C4" s="46" t="s">
-        <v>168</v>
-      </c>
-      <c r="D4" s="46" t="s">
-        <v>169</v>
-      </c>
-      <c r="E4" s="46" t="s">
+      <c r="C4" s="47" t="s">
         <v>170</v>
       </c>
-      <c r="F4" s="46" t="s">
+      <c r="D4" s="47" t="s">
         <v>171</v>
       </c>
-      <c r="G4" s="46" t="s">
+      <c r="E4" s="47" t="s">
         <v>172</v>
       </c>
-      <c r="H4" s="46" t="s">
+      <c r="F4" s="47" t="s">
         <v>173</v>
       </c>
-      <c r="I4" s="46" t="s">
+      <c r="G4" s="47" t="s">
+        <v>174</v>
+      </c>
+      <c r="H4" s="47" t="s">
+        <v>175</v>
+      </c>
+      <c r="I4" s="47" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="C5" s="9" t="s">
-        <v>174</v>
-      </c>
-      <c r="D5" s="9">
+      <c r="C5" s="10" t="s">
+        <v>176</v>
+      </c>
+      <c r="D5" s="10">
         <v>2.5</v>
       </c>
-      <c r="E5" s="21">
+      <c r="E5" s="22">
         <v>150</v>
       </c>
-      <c r="F5" s="9" t="s">
-        <v>175</v>
-      </c>
-      <c r="G5" s="9" t="s">
+      <c r="F5" s="10" t="s">
+        <v>177</v>
+      </c>
+      <c r="G5" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="H5" s="9">
+      <c r="H5" s="10">
         <v>4</v>
       </c>
-      <c r="I5" s="9" t="s">
+      <c r="I5" s="10" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="B6" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="C6" s="13" t="s">
+      <c r="C6" s="14" t="s">
+        <v>178</v>
+      </c>
+      <c r="D6" s="14">
+        <v>2</v>
+      </c>
+      <c r="E6" s="48">
+        <v>120</v>
+      </c>
+      <c r="F6" s="14" t="s">
+        <v>179</v>
+      </c>
+      <c r="G6" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="H6" s="14">
+        <v>5</v>
+      </c>
+      <c r="I6" s="14" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="C7" s="10" t="s">
         <v>176</v>
       </c>
-      <c r="D6" s="13">
-        <v>2</v>
-      </c>
-      <c r="E6" s="47">
-        <v>120</v>
-      </c>
-      <c r="F6" s="13" t="s">
-        <v>177</v>
-      </c>
-      <c r="G6" s="13" t="s">
+      <c r="D7" s="10">
+        <v>3</v>
+      </c>
+      <c r="E7" s="22">
+        <v>180</v>
+      </c>
+      <c r="F7" s="10" t="s">
+        <v>181</v>
+      </c>
+      <c r="G7" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="H7" s="10">
+        <v>4</v>
+      </c>
+      <c r="I7" s="10" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="B8" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="D8" s="14">
+        <v>2.5</v>
+      </c>
+      <c r="E8" s="48">
+        <v>150</v>
+      </c>
+      <c r="F8" s="14" t="s">
+        <v>183</v>
+      </c>
+      <c r="G8" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="H6" s="13">
+      <c r="H8" s="14">
+        <v>4</v>
+      </c>
+      <c r="I8" s="14" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>178</v>
+      </c>
+      <c r="D9" s="10">
+        <v>2.5</v>
+      </c>
+      <c r="E9" s="22">
+        <v>140</v>
+      </c>
+      <c r="F9" s="10" t="s">
+        <v>184</v>
+      </c>
+      <c r="G9" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="H9" s="10">
         <v>5</v>
       </c>
-      <c r="I6" s="13" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>174</v>
-      </c>
-      <c r="D7" s="9">
-        <v>3</v>
-      </c>
-      <c r="E7" s="21">
-        <v>180</v>
-      </c>
-      <c r="F7" s="9" t="s">
-        <v>179</v>
-      </c>
-      <c r="G7" s="9" t="s">
-        <v>59</v>
-      </c>
-      <c r="H7" s="9">
-        <v>4</v>
-      </c>
-      <c r="I7" s="9" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="B8" s="13" t="s">
-        <v>52</v>
-      </c>
-      <c r="C8" s="13" t="s">
-        <v>174</v>
-      </c>
-      <c r="D8" s="13">
-        <v>2.5</v>
-      </c>
-      <c r="E8" s="47">
-        <v>150</v>
-      </c>
-      <c r="F8" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="G8" s="13" t="s">
-        <v>54</v>
-      </c>
-      <c r="H8" s="13">
-        <v>4</v>
-      </c>
-      <c r="I8" s="13" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="7" t="s">
-        <v>85</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="C9" s="9" t="s">
-        <v>176</v>
-      </c>
-      <c r="D9" s="9">
-        <v>2.5</v>
-      </c>
-      <c r="E9" s="21">
-        <v>140</v>
-      </c>
-      <c r="F9" s="9" t="s">
-        <v>182</v>
-      </c>
-      <c r="G9" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="H9" s="9">
-        <v>5</v>
-      </c>
-      <c r="I9" s="9" t="s">
-        <v>183</v>
+      <c r="I9" s="10" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="10" spans="7:8" x14ac:dyDescent="0.25"/>
     <row r="11" spans="7:8" x14ac:dyDescent="0.25"/>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="48" t="s">
-        <v>184</v>
+      <c r="A12" s="49" t="s">
+        <v>186</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="9" t="s">
-        <v>185</v>
-      </c>
-      <c r="B13" s="20">
+      <c r="A13" s="10" t="s">
+        <v>187</v>
+      </c>
+      <c r="B13" s="21">
         <f>COUNTA(A5:A9)</f>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="9" t="s">
-        <v>186</v>
-      </c>
-      <c r="B14" s="22">
+      <c r="A14" s="10" t="s">
+        <v>188</v>
+      </c>
+      <c r="B14" s="23">
         <f>SUM(E5:E9)</f>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="9" t="s">
-        <v>187</v>
-      </c>
-      <c r="B15" s="22">
+      <c r="A15" s="10" t="s">
+        <v>189</v>
+      </c>
+      <c r="B15" s="23">
         <f>IF(B13=0,0,B14/B13)</f>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" s="9" t="s">
-        <v>188</v>
-      </c>
-      <c r="B16" s="20">
+      <c r="A16" s="10" t="s">
+        <v>190</v>
+      </c>
+      <c r="B16" s="21">
         <f>IF(B13=0,0,AVERAGE(D5:D9))</f>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="9" t="s">
-        <v>189</v>
-      </c>
-      <c r="B17" s="22">
+      <c r="A17" s="10" t="s">
+        <v>191</v>
+      </c>
+      <c r="B17" s="23">
         <f>IF(B16=0,0,B15/B16)</f>
       </c>
     </row>

</xml_diff>